<commit_message>
update excel && create readme.md
</commit_message>
<xml_diff>
--- a/matches.xlsx
+++ b/matches.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JH\code\badmintonAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEE26F1-E3D0-4A90-B7D7-14DDAE2122C3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721CBB19-EA23-4CB1-BFD9-A194E15DCE99}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="重大赛事" sheetId="1" r:id="rId1"/>
@@ -4743,6 +4743,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>